<commit_message>
Update agent metadata and regenerate payables preview reports
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/.agents/outputs/vb-payables-preview/live-payables-preview.xlsx
+++ b/.agents/outputs/vb-payables-preview/live-payables-preview.xlsx
@@ -438,7 +438,7 @@
         <v>Generated</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-10-04T16:43:20.136Z</v>
+        <v>2026-10-04T17:12:22.215Z</v>
       </c>
     </row>
     <row r="5">
@@ -700,7 +700,7 @@
         <v>Generated</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-10-04T16:43:20.136Z</v>
+        <v>2026-10-04T17:12:22.215Z</v>
       </c>
     </row>
     <row r="3">
@@ -1258,7 +1258,7 @@
         <v>Generated</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-10-04T16:43:20.136Z</v>
+        <v>2026-10-04T17:12:22.215Z</v>
       </c>
     </row>
     <row r="3">
@@ -1434,7 +1434,7 @@
         <v>Generated</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-10-04T16:43:20.136Z</v>
+        <v>2026-10-04T17:12:22.215Z</v>
       </c>
     </row>
     <row r="3">
@@ -1697,7 +1697,7 @@
         <v>Generated</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-10-04T16:43:20.136Z</v>
+        <v>2026-10-04T17:12:22.215Z</v>
       </c>
     </row>
     <row r="3">
@@ -1786,7 +1786,7 @@
         <v>Generated</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-10-04T16:43:20.136Z</v>
+        <v>2026-10-04T17:12:22.215Z</v>
       </c>
     </row>
     <row r="3">

</xml_diff>